<commit_message>
working 2D stranded coil planar
</commit_message>
<xml_diff>
--- a/tests/coil_2D_ave/input_template.xlsx
+++ b/tests/coil_2D_ave/input_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="element_types"/>
@@ -371,7 +371,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -382,12 +382,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -419,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -449,9 +443,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1091,7 +1082,7 @@
     <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>101</v>
       </c>
@@ -1099,15 +1090,15 @@
         <v>102</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="11">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -1513,7 +1504,7 @@
         <v>50</v>
       </c>
       <c r="K2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" s="1">
         <v>0</v>

</xml_diff>